<commit_message>
feat: add DAO execution area and statistics
</commit_message>
<xml_diff>
--- a/public/SIGA-modelo-atualizacao.xlsx
+++ b/public/SIGA-modelo-atualizacao.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demandas" sheetId="1" r:id="R5d05c6139ddf42c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pessoas" sheetId="2" r:id="R69adcf05154f408d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="3" r:id="R52338a81093c4758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demandas" sheetId="1" r:id="Rf2a04d3709854476"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pessoas" sheetId="2" r:id="R6f703f9dd07f41e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="3" r:id="Rc71a1cb1626f4c3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -853,7 +853,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="E2:E21">
-      <x:formula1>"SLC,SAP,SME,AE"</x:formula1>
+      <x:formula1>"DAO,SLC,SAP,SME,AE"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="G2:G21">
       <x:formula1>"SIM,NÃO"</x:formula1>
@@ -916,7 +916,7 @@
         <x:v>5. Valores permitidos</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>Prioridade: BAIXA, MEDIA, ALTA (vazio somente em triagem). Seção: SLC, SAP, SME, AE. Ativo: SIM ou NÃO.</x:v>
+        <x:v>Prioridade: BAIXA, MEDIA, ALTA (vazio somente em triagem). Seção: DAO, SLC, SAP, SME, AE. Ativo: SIM ou NÃO.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="52" customHeight="1">

</xml_diff>